<commit_message>
Publish LeeValley_2023_WCH, LiptovskyMikulas_2018_WC, Markkleeberg_2021_WC, Prague_2019_WC
</commit_message>
<xml_diff>
--- a/events/LeeValley_2023_WCH/LeeValley_2023_WCH_start.xlsx
+++ b/events/LeeValley_2023_WCH/LeeValley_2023_WCH_start.xlsx
@@ -50084,6 +50084,11 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
+      <c r="X815" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
     </row>
     <row r="816">
       <c r="A816" t="inlineStr">

</xml_diff>